<commit_message>
Update CoMET code and ablation experiments
</commit_message>
<xml_diff>
--- a/output1/XGBoost_val_predictions.xlsx
+++ b/output1/XGBoost_val_predictions.xlsx
@@ -824,7 +824,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>3.868421052631578</v>
+        <v>3.868421052631577</v>
       </c>
       <c r="H13" t="n">
         <v>0.141230434179306</v>
@@ -2057,7 +2057,7 @@
         <v>4.888268156424582</v>
       </c>
       <c r="H54" t="n">
-        <v>0.08633526414632797</v>
+        <v>0.07159017026424408</v>
       </c>
     </row>
     <row r="55">
@@ -2087,7 +2087,7 @@
         <v>2.067039106145252</v>
       </c>
       <c r="H55" t="n">
-        <v>0.4093947410583496</v>
+        <v>0.3944685161113739</v>
       </c>
     </row>
     <row r="56">
@@ -2117,7 +2117,7 @@
         <v>9.441340782122904</v>
       </c>
       <c r="H56" t="n">
-        <v>0.08586271852254868</v>
+        <v>0.1360622048377991</v>
       </c>
     </row>
     <row r="57">
@@ -2147,7 +2147,7 @@
         <v>4.804469273743017</v>
       </c>
       <c r="H57" t="n">
-        <v>0.06175263971090317</v>
+        <v>0.07427048683166504</v>
       </c>
     </row>
     <row r="58">
@@ -2177,7 +2177,7 @@
         <v>4.329608938547486</v>
       </c>
       <c r="H58" t="n">
-        <v>0.0197158195078373</v>
+        <v>0.01994129084050655</v>
       </c>
     </row>
     <row r="59">
@@ -2207,7 +2207,7 @@
         <v>9.441340782122904</v>
       </c>
       <c r="H59" t="n">
-        <v>0.004490358289331198</v>
+        <v>0.006425484083592892</v>
       </c>
     </row>
     <row r="60">
@@ -2237,7 +2237,7 @@
         <v>4.189944134078212</v>
       </c>
       <c r="H60" t="n">
-        <v>0.07548834383487701</v>
+        <v>0.1675331890583038</v>
       </c>
     </row>
     <row r="61">
@@ -2267,7 +2267,7 @@
         <v>5.363128491620112</v>
       </c>
       <c r="H61" t="n">
-        <v>0.151056706905365</v>
+        <v>0.1442763954401016</v>
       </c>
     </row>
     <row r="62">
@@ -2297,7 +2297,7 @@
         <v>21.08938547486034</v>
       </c>
       <c r="H62" t="n">
-        <v>0.845198929309845</v>
+        <v>0.8302593231201172</v>
       </c>
     </row>
     <row r="63">
@@ -2327,7 +2327,7 @@
         <v>28.46368715083799</v>
       </c>
       <c r="H63" t="n">
-        <v>0.9910116195678711</v>
+        <v>0.994787335395813</v>
       </c>
     </row>
     <row r="64">
@@ -2357,7 +2357,7 @@
         <v>14.41340782122905</v>
       </c>
       <c r="H64" t="n">
-        <v>0.5222093462944031</v>
+        <v>0.5174112319946289</v>
       </c>
     </row>
     <row r="65">
@@ -2387,7 +2387,7 @@
         <v>25.19553072625699</v>
       </c>
       <c r="H65" t="n">
-        <v>0.9260798096656799</v>
+        <v>0.8517318964004517</v>
       </c>
     </row>
     <row r="66">
@@ -2417,7 +2417,7 @@
         <v>7.765363128491621</v>
       </c>
       <c r="H66" t="n">
-        <v>0.07261195033788681</v>
+        <v>0.08983442187309265</v>
       </c>
     </row>
     <row r="67">
@@ -2447,7 +2447,7 @@
         <v>16.36871508379888</v>
       </c>
       <c r="H67" t="n">
-        <v>0.9280277490615845</v>
+        <v>0.9150273203849792</v>
       </c>
     </row>
     <row r="68">
@@ -4277,7 +4277,7 @@
         <v>0.8947368421052632</v>
       </c>
       <c r="H128" t="n">
-        <v>0.279352068901062</v>
+        <v>0.3209025859832764</v>
       </c>
     </row>
     <row r="129">
@@ -4307,7 +4307,7 @@
         <v>1.157894736842105</v>
       </c>
       <c r="H129" t="n">
-        <v>0.05609889701008797</v>
+        <v>0.06881771981716156</v>
       </c>
     </row>
     <row r="130">
@@ -4337,7 +4337,7 @@
         <v>1.105263157894737</v>
       </c>
       <c r="H130" t="n">
-        <v>0.5627781748771667</v>
+        <v>0.3801042139530182</v>
       </c>
     </row>
     <row r="131">
@@ -4367,7 +4367,7 @@
         <v>1.921052631578948</v>
       </c>
       <c r="H131" t="n">
-        <v>0.6440984606742859</v>
+        <v>0.6641471385955811</v>
       </c>
     </row>
     <row r="132">
@@ -4397,7 +4397,7 @@
         <v>0.6578947368421053</v>
       </c>
       <c r="H132" t="n">
-        <v>0.3110570907592773</v>
+        <v>0.4068426191806793</v>
       </c>
     </row>
     <row r="133">
@@ -4427,7 +4427,7 @@
         <v>0.1052631578947368</v>
       </c>
       <c r="H133" t="n">
-        <v>0.600288987159729</v>
+        <v>0.6395171880722046</v>
       </c>
     </row>
     <row r="134">
@@ -4457,7 +4457,7 @@
         <v>1.526315789473684</v>
       </c>
       <c r="H134" t="n">
-        <v>0.2642364501953125</v>
+        <v>0.199347585439682</v>
       </c>
     </row>
     <row r="135">
@@ -4487,7 +4487,7 @@
         <v>0.631578947368421</v>
       </c>
       <c r="H135" t="n">
-        <v>0.7307234406471252</v>
+        <v>0.5480759143829346</v>
       </c>
     </row>
     <row r="136">
@@ -4517,7 +4517,7 @@
         <v>1.789473684210526</v>
       </c>
       <c r="H136" t="n">
-        <v>0.09612832963466644</v>
+        <v>0.1203828752040863</v>
       </c>
     </row>
     <row r="137">
@@ -4547,7 +4547,7 @@
         <v>1.447368421052632</v>
       </c>
       <c r="H137" t="n">
-        <v>0.06360390782356262</v>
+        <v>0.05866758897900581</v>
       </c>
     </row>
     <row r="138">
@@ -4577,7 +4577,7 @@
         <v>4.657894736842105</v>
       </c>
       <c r="H138" t="n">
-        <v>0.1405435800552368</v>
+        <v>0.1484376043081284</v>
       </c>
     </row>
     <row r="139">
@@ -4607,7 +4607,7 @@
         <v>1.710526315789474</v>
       </c>
       <c r="H139" t="n">
-        <v>0.05638320744037628</v>
+        <v>0.09537980705499649</v>
       </c>
     </row>
     <row r="140">
@@ -4637,7 +4637,7 @@
         <v>1.368421052631579</v>
       </c>
       <c r="H140" t="n">
-        <v>0.4144608378410339</v>
+        <v>0.4337477684020996</v>
       </c>
     </row>
     <row r="141">
@@ -4667,7 +4667,7 @@
         <v>2.763157894736842</v>
       </c>
       <c r="H141" t="n">
-        <v>0.9628447890281677</v>
+        <v>0.9586783647537231</v>
       </c>
     </row>
     <row r="142">
@@ -4697,7 +4697,7 @@
         <v>1.131578947368421</v>
       </c>
       <c r="H142" t="n">
-        <v>0.2673699557781219</v>
+        <v>0.2530069351196289</v>
       </c>
     </row>
     <row r="143">
@@ -4727,7 +4727,7 @@
         <v>1.552631578947368</v>
       </c>
       <c r="H143" t="n">
-        <v>0.1567145735025406</v>
+        <v>0.1366015821695328</v>
       </c>
     </row>
     <row r="144">
@@ -4757,7 +4757,7 @@
         <v>1.368421052631579</v>
       </c>
       <c r="H144" t="n">
-        <v>0.02248295955359936</v>
+        <v>0.03643666207790375</v>
       </c>
     </row>
     <row r="145">
@@ -4787,7 +4787,7 @@
         <v>0.9736842105263158</v>
       </c>
       <c r="H145" t="n">
-        <v>0.08955033123493195</v>
+        <v>0.07379965484142303</v>
       </c>
     </row>
     <row r="146">
@@ -4817,7 +4817,7 @@
         <v>0.7368421052631579</v>
       </c>
       <c r="H146" t="n">
-        <v>0.2613202035427094</v>
+        <v>0.2218724340200424</v>
       </c>
     </row>
     <row r="147">
@@ -4847,7 +4847,7 @@
         <v>1.684210526315789</v>
       </c>
       <c r="H147" t="n">
-        <v>0.6138044595718384</v>
+        <v>0.5695863962173462</v>
       </c>
     </row>
     <row r="148">
@@ -4877,7 +4877,7 @@
         <v>1.947368421052632</v>
       </c>
       <c r="H148" t="n">
-        <v>0.199267640709877</v>
+        <v>0.2416257411241531</v>
       </c>
     </row>
     <row r="149">
@@ -4907,7 +4907,7 @@
         <v>1.078947368421053</v>
       </c>
       <c r="H149" t="n">
-        <v>0.4329874217510223</v>
+        <v>0.4776633977890015</v>
       </c>
     </row>
     <row r="150">
@@ -4937,7 +4937,7 @@
         <v>0.8947368421052632</v>
       </c>
       <c r="H150" t="n">
-        <v>0.04093195125460625</v>
+        <v>0.03519907966256142</v>
       </c>
     </row>
     <row r="151">
@@ -4967,7 +4967,7 @@
         <v>1.631578947368421</v>
       </c>
       <c r="H151" t="n">
-        <v>0.1238379329442978</v>
+        <v>0.1424771100282669</v>
       </c>
     </row>
     <row r="152">
@@ -4997,7 +4997,7 @@
         <v>1.789473684210526</v>
       </c>
       <c r="H152" t="n">
-        <v>0.274746298789978</v>
+        <v>0.4849015176296234</v>
       </c>
     </row>
     <row r="153">
@@ -5027,7 +5027,7 @@
         <v>0.9473684210526316</v>
       </c>
       <c r="H153" t="n">
-        <v>0.7437765002250671</v>
+        <v>0.7381154894828796</v>
       </c>
     </row>
     <row r="154">
@@ -5057,7 +5057,7 @@
         <v>1.868421052631579</v>
       </c>
       <c r="H154" t="n">
-        <v>0.238520622253418</v>
+        <v>0.2033255696296692</v>
       </c>
     </row>
     <row r="155">
@@ -5087,7 +5087,7 @@
         <v>2.5</v>
       </c>
       <c r="H155" t="n">
-        <v>0.3432484865188599</v>
+        <v>0.2431909143924713</v>
       </c>
     </row>
     <row r="156">
@@ -5117,7 +5117,7 @@
         <v>0.5789473684210527</v>
       </c>
       <c r="H156" t="n">
-        <v>0.005025149323046207</v>
+        <v>0.006227055564522743</v>
       </c>
     </row>
     <row r="157">
@@ -5147,7 +5147,7 @@
         <v>1.184210526315789</v>
       </c>
       <c r="H157" t="n">
-        <v>0.04317962750792503</v>
+        <v>0.07621835172176361</v>
       </c>
     </row>
     <row r="158">
@@ -5177,7 +5177,7 @@
         <v>8.631578947368421</v>
       </c>
       <c r="H158" t="n">
-        <v>0.4059996604919434</v>
+        <v>0.5666489005088806</v>
       </c>
     </row>
     <row r="159">
@@ -5207,7 +5207,7 @@
         <v>0.7894736842105263</v>
       </c>
       <c r="H159" t="n">
-        <v>0.345408707857132</v>
+        <v>0.2851996123790741</v>
       </c>
     </row>
     <row r="160">
@@ -5237,7 +5237,7 @@
         <v>54.6578947368421</v>
       </c>
       <c r="H160" t="n">
-        <v>0.3696103692054749</v>
+        <v>0.3175185918807983</v>
       </c>
     </row>
     <row r="161">
@@ -5267,7 +5267,7 @@
         <v>1.578947368421053</v>
       </c>
       <c r="H161" t="n">
-        <v>0.1216223686933517</v>
+        <v>0.2094737589359283</v>
       </c>
     </row>
     <row r="162">
@@ -5297,7 +5297,7 @@
         <v>4.789473684210527</v>
       </c>
       <c r="H162" t="n">
-        <v>0.1782027333974838</v>
+        <v>0.08130070567131042</v>
       </c>
     </row>
     <row r="163">
@@ -5327,7 +5327,7 @@
         <v>0.6052631578947368</v>
       </c>
       <c r="H163" t="n">
-        <v>0.7792239785194397</v>
+        <v>0.8849528431892395</v>
       </c>
     </row>
     <row r="164">
@@ -5357,7 +5357,7 @@
         <v>5.315789473684211</v>
       </c>
       <c r="H164" t="n">
-        <v>0.1419511139392853</v>
+        <v>0.06319513916969299</v>
       </c>
     </row>
     <row r="165">
@@ -5387,7 +5387,7 @@
         <v>41.21052631578947</v>
       </c>
       <c r="H165" t="n">
-        <v>0.9803440570831299</v>
+        <v>0.9653216004371643</v>
       </c>
     </row>
     <row r="166">
@@ -5417,7 +5417,7 @@
         <v>5.289473684210527</v>
       </c>
       <c r="H166" t="n">
-        <v>0.05807341262698174</v>
+        <v>0.05954854190349579</v>
       </c>
     </row>
     <row r="167">
@@ -5447,7 +5447,7 @@
         <v>9</v>
       </c>
       <c r="H167" t="n">
-        <v>0.8957365751266479</v>
+        <v>0.8114169239997864</v>
       </c>
     </row>
     <row r="168">
@@ -5477,7 +5477,7 @@
         <v>3.5</v>
       </c>
       <c r="H168" t="n">
-        <v>0.5660029649734497</v>
+        <v>0.479361891746521</v>
       </c>
     </row>
     <row r="169">
@@ -5507,7 +5507,7 @@
         <v>1.526315789473684</v>
       </c>
       <c r="H169" t="n">
-        <v>0.07050850242376328</v>
+        <v>0.1331141144037247</v>
       </c>
     </row>
     <row r="170">
@@ -5537,7 +5537,7 @@
         <v>15.05263157894737</v>
       </c>
       <c r="H170" t="n">
-        <v>0.7292978167533875</v>
+        <v>0.804141104221344</v>
       </c>
     </row>
     <row r="171">
@@ -5567,7 +5567,7 @@
         <v>8.631578947368421</v>
       </c>
       <c r="H171" t="n">
-        <v>0.9674578905105591</v>
+        <v>0.9554672837257385</v>
       </c>
     </row>
     <row r="172">
@@ -5597,7 +5597,7 @@
         <v>0.2631578947368421</v>
       </c>
       <c r="H172" t="n">
-        <v>0.4243386387825012</v>
+        <v>0.4479626715183258</v>
       </c>
     </row>
     <row r="173">
@@ -5627,7 +5627,7 @@
         <v>0.4736842105263157</v>
       </c>
       <c r="H173" t="n">
-        <v>0.03173608705401421</v>
+        <v>0.06222037598490715</v>
       </c>
     </row>
     <row r="174">
@@ -5657,7 +5657,7 @@
         <v>1.684210526315789</v>
       </c>
       <c r="H174" t="n">
-        <v>0.01372931059449911</v>
+        <v>0.04765965044498444</v>
       </c>
     </row>
     <row r="175">
@@ -5687,7 +5687,7 @@
         <v>7.710526315789473</v>
       </c>
       <c r="H175" t="n">
-        <v>0.1240770295262337</v>
+        <v>0.1903188675642014</v>
       </c>
     </row>
     <row r="176">
@@ -5717,7 +5717,7 @@
         <v>0.4473684210526316</v>
       </c>
       <c r="H176" t="n">
-        <v>0.9356585144996643</v>
+        <v>0.905428946018219</v>
       </c>
     </row>
     <row r="177">
@@ -5747,7 +5747,7 @@
         <v>55.71052631578947</v>
       </c>
       <c r="H177" t="n">
-        <v>0.7445886731147766</v>
+        <v>0.6812742948532104</v>
       </c>
     </row>
     <row r="178">
@@ -5777,7 +5777,7 @@
         <v>7.342105263157895</v>
       </c>
       <c r="H178" t="n">
-        <v>0.1384412050247192</v>
+        <v>0.1680590659379959</v>
       </c>
     </row>
     <row r="179">
@@ -5807,7 +5807,7 @@
         <v>17.07894736842105</v>
       </c>
       <c r="H179" t="n">
-        <v>0.1567575186491013</v>
+        <v>0.1685015261173248</v>
       </c>
     </row>
     <row r="180">
@@ -5837,7 +5837,7 @@
         <v>9.441340782122904</v>
       </c>
       <c r="H180" t="n">
-        <v>0.1806812137365341</v>
+        <v>0.2013924866914749</v>
       </c>
     </row>
     <row r="181">
@@ -5867,7 +5867,7 @@
         <v>9.441340782122904</v>
       </c>
       <c r="H181" t="n">
-        <v>0.09071965515613556</v>
+        <v>0.09406254440546036</v>
       </c>
     </row>
     <row r="182">
@@ -5897,7 +5897,7 @@
         <v>17.40223463687151</v>
       </c>
       <c r="H182" t="n">
-        <v>0.8230205178260803</v>
+        <v>0.8257396221160889</v>
       </c>
     </row>
     <row r="183">
@@ -5927,7 +5927,7 @@
         <v>9.441340782122904</v>
       </c>
       <c r="H183" t="n">
-        <v>0.03773145377635956</v>
+        <v>0.04290968552231789</v>
       </c>
     </row>
     <row r="184">
@@ -5957,7 +5957,7 @@
         <v>7.178770949720671</v>
       </c>
       <c r="H184" t="n">
-        <v>0.9371609091758728</v>
+        <v>0.9384148716926575</v>
       </c>
     </row>
     <row r="185">
@@ -5987,7 +5987,7 @@
         <v>7.011173184357543</v>
       </c>
       <c r="H185" t="n">
-        <v>0.08073617517948151</v>
+        <v>0.09125663340091705</v>
       </c>
     </row>
     <row r="186">
@@ -6017,7 +6017,7 @@
         <v>11.95530726256983</v>
       </c>
       <c r="H186" t="n">
-        <v>0.4130034148693085</v>
+        <v>0.4233327805995941</v>
       </c>
     </row>
     <row r="187">
@@ -6047,7 +6047,7 @@
         <v>0.6983240223463688</v>
       </c>
       <c r="H187" t="n">
-        <v>0.9037432670593262</v>
+        <v>0.9145841598510742</v>
       </c>
     </row>
     <row r="188">
@@ -6077,7 +6077,7 @@
         <v>46.08938547486034</v>
       </c>
       <c r="H188" t="n">
-        <v>0.957854688167572</v>
+        <v>0.958606481552124</v>
       </c>
     </row>
     <row r="189">
@@ -6107,7 +6107,7 @@
         <v>2.067039106145252</v>
       </c>
       <c r="H189" t="n">
-        <v>0.1658321768045425</v>
+        <v>0.1563675999641418</v>
       </c>
     </row>
     <row r="190">
@@ -6137,7 +6137,7 @@
         <v>35.81005586592179</v>
       </c>
       <c r="H190" t="n">
-        <v>0.9506920576095581</v>
+        <v>0.9472966194152832</v>
       </c>
     </row>
     <row r="191">
@@ -6167,7 +6167,7 @@
         <v>7.178770949720671</v>
       </c>
       <c r="H191" t="n">
-        <v>0.1157115548849106</v>
+        <v>0.1201271712779999</v>
       </c>
     </row>
     <row r="192">
@@ -6197,7 +6197,7 @@
         <v>6.843575418994414</v>
       </c>
       <c r="H192" t="n">
-        <v>0.9510862231254578</v>
+        <v>0.9477163553237915</v>
       </c>
     </row>
     <row r="193">
@@ -6227,7 +6227,7 @@
         <v>1.871508379888268</v>
       </c>
       <c r="H193" t="n">
-        <v>0.5095195174217224</v>
+        <v>0.5201552510261536</v>
       </c>
     </row>
     <row r="194">
@@ -6257,7 +6257,7 @@
         <v>18</v>
       </c>
       <c r="H194" t="n">
-        <v>0.2054219990968704</v>
+        <v>0.1216402873396873</v>
       </c>
     </row>
     <row r="195">
@@ -6287,7 +6287,7 @@
         <v>8</v>
       </c>
       <c r="H195" t="n">
-        <v>0.1481262743473053</v>
+        <v>0.1916322261095047</v>
       </c>
     </row>
     <row r="196">
@@ -6317,7 +6317,7 @@
         <v>18</v>
       </c>
       <c r="H196" t="n">
-        <v>0.5386888980865479</v>
+        <v>0.62935870885849</v>
       </c>
     </row>
     <row r="197">
@@ -6347,7 +6347,7 @@
         <v>2</v>
       </c>
       <c r="H197" t="n">
-        <v>0.1072991937398911</v>
+        <v>0.0998668447136879</v>
       </c>
     </row>
     <row r="198">
@@ -6377,7 +6377,7 @@
         <v>8</v>
       </c>
       <c r="H198" t="n">
-        <v>0.02045959234237671</v>
+        <v>0.01414178032428026</v>
       </c>
     </row>
     <row r="199">
@@ -6407,7 +6407,7 @@
         <v>9</v>
       </c>
       <c r="H199" t="n">
-        <v>0.03837417438626289</v>
+        <v>0.06820062547922134</v>
       </c>
     </row>
     <row r="200">
@@ -6437,7 +6437,7 @@
         <v>21</v>
       </c>
       <c r="H200" t="n">
-        <v>0.09689842164516449</v>
+        <v>0.1051014140248299</v>
       </c>
     </row>
     <row r="201">
@@ -6467,7 +6467,7 @@
         <v>8</v>
       </c>
       <c r="H201" t="n">
-        <v>0.03173056244850159</v>
+        <v>0.02213819324970245</v>
       </c>
     </row>
     <row r="202">
@@ -6497,7 +6497,7 @@
         <v>5</v>
       </c>
       <c r="H202" t="n">
-        <v>0.0285334624350071</v>
+        <v>0.02233624272048473</v>
       </c>
     </row>
     <row r="203">
@@ -6527,7 +6527,7 @@
         <v>8</v>
       </c>
       <c r="H203" t="n">
-        <v>0.03802888095378876</v>
+        <v>0.05035967752337456</v>
       </c>
     </row>
     <row r="204">
@@ -6557,7 +6557,7 @@
         <v>2</v>
       </c>
       <c r="H204" t="n">
-        <v>0.1361658424139023</v>
+        <v>0.1035895794630051</v>
       </c>
     </row>
     <row r="205">
@@ -6587,7 +6587,7 @@
         <v>20</v>
       </c>
       <c r="H205" t="n">
-        <v>0.5573458671569824</v>
+        <v>0.6299346685409546</v>
       </c>
     </row>
     <row r="206">
@@ -6617,7 +6617,7 @@
         <v>5</v>
       </c>
       <c r="H206" t="n">
-        <v>0.05452590063214302</v>
+        <v>0.07639003545045853</v>
       </c>
     </row>
     <row r="207">
@@ -6647,7 +6647,7 @@
         <v>8</v>
       </c>
       <c r="H207" t="n">
-        <v>0.5898982286453247</v>
+        <v>0.5613998174667358</v>
       </c>
     </row>
     <row r="208">
@@ -6677,7 +6677,7 @@
         <v>1</v>
       </c>
       <c r="H208" t="n">
-        <v>0.009387915022671223</v>
+        <v>0.004899866878986359</v>
       </c>
     </row>
     <row r="209">
@@ -6707,7 +6707,7 @@
         <v>8</v>
       </c>
       <c r="H209" t="n">
-        <v>0.01491502858698368</v>
+        <v>0.01836766488850117</v>
       </c>
     </row>
     <row r="210">
@@ -6737,7 +6737,7 @@
         <v>13</v>
       </c>
       <c r="H210" t="n">
-        <v>0.01972928456962109</v>
+        <v>0.07217880338430405</v>
       </c>
     </row>
     <row r="211">
@@ -6767,7 +6767,7 @@
         <v>2</v>
       </c>
       <c r="H211" t="n">
-        <v>0.1150989085435867</v>
+        <v>0.1811566203832626</v>
       </c>
     </row>
     <row r="212">
@@ -6797,7 +6797,7 @@
         <v>7</v>
       </c>
       <c r="H212" t="n">
-        <v>0.08098970353603363</v>
+        <v>0.06444508582353592</v>
       </c>
     </row>
     <row r="213">
@@ -6827,7 +6827,7 @@
         <v>7</v>
       </c>
       <c r="H213" t="n">
-        <v>0.1070469096302986</v>
+        <v>0.1089436635375023</v>
       </c>
     </row>
     <row r="214">
@@ -6857,7 +6857,7 @@
         <v>2</v>
       </c>
       <c r="H214" t="n">
-        <v>0.03917770087718964</v>
+        <v>0.02824223227798939</v>
       </c>
     </row>
     <row r="215">
@@ -6887,7 +6887,7 @@
         <v>8</v>
       </c>
       <c r="H215" t="n">
-        <v>0.5388913154602051</v>
+        <v>0.3932392597198486</v>
       </c>
     </row>
     <row r="216">
@@ -6917,7 +6917,7 @@
         <v>6</v>
       </c>
       <c r="H216" t="n">
-        <v>0.01885375380516052</v>
+        <v>0.01230619195848703</v>
       </c>
     </row>
     <row r="217">
@@ -6947,7 +6947,7 @@
         <v>8</v>
       </c>
       <c r="H217" t="n">
-        <v>0.03261655196547508</v>
+        <v>0.04318934306502342</v>
       </c>
     </row>
     <row r="218">
@@ -6977,7 +6977,7 @@
         <v>8</v>
       </c>
       <c r="H218" t="n">
-        <v>0.08450522273778915</v>
+        <v>0.134812593460083</v>
       </c>
     </row>
     <row r="219">
@@ -7007,7 +7007,7 @@
         <v>8</v>
       </c>
       <c r="H219" t="n">
-        <v>0.1754961162805557</v>
+        <v>0.1313362568616867</v>
       </c>
     </row>
     <row r="220">
@@ -7037,7 +7037,7 @@
         <v>14</v>
       </c>
       <c r="H220" t="n">
-        <v>0.00708024250343442</v>
+        <v>0.0110944090411067</v>
       </c>
     </row>
     <row r="221">
@@ -7067,7 +7067,7 @@
         <v>5</v>
       </c>
       <c r="H221" t="n">
-        <v>0.05558884143829346</v>
+        <v>0.09115880727767944</v>
       </c>
     </row>
     <row r="222">
@@ -7097,7 +7097,7 @@
         <v>20</v>
       </c>
       <c r="H222" t="n">
-        <v>0.247226744890213</v>
+        <v>0.08646408468484879</v>
       </c>
     </row>
     <row r="223">
@@ -7127,7 +7127,7 @@
         <v>3</v>
       </c>
       <c r="H223" t="n">
-        <v>0.1231515556573868</v>
+        <v>0.08383473753929138</v>
       </c>
     </row>
     <row r="224">
@@ -7157,7 +7157,7 @@
         <v>8</v>
       </c>
       <c r="H224" t="n">
-        <v>0.315434068441391</v>
+        <v>0.1612402945756912</v>
       </c>
     </row>
     <row r="225">
@@ -7187,7 +7187,7 @@
         <v>17</v>
       </c>
       <c r="H225" t="n">
-        <v>0.09258683770895004</v>
+        <v>0.1227694675326347</v>
       </c>
     </row>
     <row r="226">
@@ -7217,7 +7217,7 @@
         <v>12</v>
       </c>
       <c r="H226" t="n">
-        <v>0.04368069395422935</v>
+        <v>0.05509324744343758</v>
       </c>
     </row>
     <row r="227">
@@ -7247,7 +7247,7 @@
         <v>5</v>
       </c>
       <c r="H227" t="n">
-        <v>0.1587750166654587</v>
+        <v>0.1477107852697372</v>
       </c>
     </row>
     <row r="228">
@@ -7277,7 +7277,7 @@
         <v>7</v>
       </c>
       <c r="H228" t="n">
-        <v>0.03041830100119114</v>
+        <v>0.0146580608561635</v>
       </c>
     </row>
     <row r="229">
@@ -7307,7 +7307,7 @@
         <v>14</v>
       </c>
       <c r="H229" t="n">
-        <v>0.7579120993614197</v>
+        <v>0.7201489210128784</v>
       </c>
     </row>
     <row r="230">
@@ -7337,7 +7337,7 @@
         <v>12</v>
       </c>
       <c r="H230" t="n">
-        <v>0.1453185826539993</v>
+        <v>0.1275037378072739</v>
       </c>
     </row>
     <row r="231">
@@ -7367,7 +7367,7 @@
         <v>8</v>
       </c>
       <c r="H231" t="n">
-        <v>0.5698209404945374</v>
+        <v>0.5525283217430115</v>
       </c>
     </row>
     <row r="232">
@@ -7397,7 +7397,7 @@
         <v>4</v>
       </c>
       <c r="H232" t="n">
-        <v>0.3104065358638763</v>
+        <v>0.3585453033447266</v>
       </c>
     </row>
     <row r="233">
@@ -7427,7 +7427,7 @@
         <v>6</v>
       </c>
       <c r="H233" t="n">
-        <v>0.07628533989191055</v>
+        <v>0.1381048411130905</v>
       </c>
     </row>
     <row r="234">
@@ -7457,7 +7457,7 @@
         <v>18</v>
       </c>
       <c r="H234" t="n">
-        <v>0.8188061118125916</v>
+        <v>0.8816850185394287</v>
       </c>
     </row>
     <row r="235">
@@ -7487,7 +7487,7 @@
         <v>8</v>
       </c>
       <c r="H235" t="n">
-        <v>0.09025175869464874</v>
+        <v>0.09519543498754501</v>
       </c>
     </row>
     <row r="236">
@@ -7517,7 +7517,7 @@
         <v>18</v>
       </c>
       <c r="H236" t="n">
-        <v>0.1673406809568405</v>
+        <v>0.322479248046875</v>
       </c>
     </row>
     <row r="237">
@@ -7547,7 +7547,7 @@
         <v>35</v>
       </c>
       <c r="H237" t="n">
-        <v>0.8752765655517578</v>
+        <v>0.9106444716453552</v>
       </c>
     </row>
     <row r="238">
@@ -7577,7 +7577,7 @@
         <v>5</v>
       </c>
       <c r="H238" t="n">
-        <v>0.08189087361097336</v>
+        <v>0.1502008736133575</v>
       </c>
     </row>
     <row r="239">
@@ -7607,7 +7607,7 @@
         <v>3</v>
       </c>
       <c r="H239" t="n">
-        <v>0.07894949615001678</v>
+        <v>0.07412987947463989</v>
       </c>
     </row>
     <row r="240">
@@ -7637,7 +7637,7 @@
         <v>22</v>
       </c>
       <c r="H240" t="n">
-        <v>0.1231897100806236</v>
+        <v>0.2445693165063858</v>
       </c>
     </row>
     <row r="241">
@@ -7667,7 +7667,7 @@
         <v>8</v>
       </c>
       <c r="H241" t="n">
-        <v>0.0205481331795454</v>
+        <v>0.01941570639610291</v>
       </c>
     </row>
     <row r="242">
@@ -7697,7 +7697,7 @@
         <v>15</v>
       </c>
       <c r="H242" t="n">
-        <v>0.7234095335006714</v>
+        <v>0.8783669471740723</v>
       </c>
     </row>
     <row r="243">
@@ -7727,7 +7727,7 @@
         <v>14</v>
       </c>
       <c r="H243" t="n">
-        <v>0.3103893399238586</v>
+        <v>0.2521602213382721</v>
       </c>
     </row>
     <row r="244">
@@ -7757,7 +7757,7 @@
         <v>10</v>
       </c>
       <c r="H244" t="n">
-        <v>0.1717826724052429</v>
+        <v>0.2493603825569153</v>
       </c>
     </row>
     <row r="245">
@@ -7787,7 +7787,7 @@
         <v>14</v>
       </c>
       <c r="H245" t="n">
-        <v>0.8463157415390015</v>
+        <v>0.7578557729721069</v>
       </c>
     </row>
     <row r="246">
@@ -7817,7 +7817,7 @@
         <v>17</v>
       </c>
       <c r="H246" t="n">
-        <v>0.1638559252023697</v>
+        <v>0.1053895875811577</v>
       </c>
     </row>
     <row r="247">
@@ -7847,7 +7847,7 @@
         <v>6</v>
       </c>
       <c r="H247" t="n">
-        <v>0.1457552015781403</v>
+        <v>0.1675548702478409</v>
       </c>
     </row>
     <row r="248">
@@ -7877,7 +7877,7 @@
         <v>9</v>
       </c>
       <c r="H248" t="n">
-        <v>0.2216087132692337</v>
+        <v>0.1929022520780563</v>
       </c>
     </row>
     <row r="249">
@@ -7907,7 +7907,7 @@
         <v>8</v>
       </c>
       <c r="H249" t="n">
-        <v>0.3778042197227478</v>
+        <v>0.374346911907196</v>
       </c>
     </row>
     <row r="250">
@@ -7937,7 +7937,7 @@
         <v>8</v>
       </c>
       <c r="H250" t="n">
-        <v>0.03163796663284302</v>
+        <v>0.0301357377320528</v>
       </c>
     </row>
     <row r="251">
@@ -7967,7 +7967,7 @@
         <v>1</v>
       </c>
       <c r="H251" t="n">
-        <v>0.03832576796412468</v>
+        <v>0.07062568515539169</v>
       </c>
     </row>
     <row r="252">
@@ -7997,7 +7997,7 @@
         <v>7</v>
       </c>
       <c r="H252" t="n">
-        <v>0.2320428788661957</v>
+        <v>0.2739134132862091</v>
       </c>
     </row>
     <row r="253">
@@ -8027,7 +8027,7 @@
         <v>7</v>
       </c>
       <c r="H253" t="n">
-        <v>0.02212599106132984</v>
+        <v>0.0125660253688693</v>
       </c>
     </row>
     <row r="254">
@@ -8057,7 +8057,7 @@
         <v>1.368421052631579</v>
       </c>
       <c r="H254" t="n">
-        <v>0.6110605001449585</v>
+        <v>0.5813892483711243</v>
       </c>
     </row>
     <row r="255">
@@ -8087,7 +8087,7 @@
         <v>1.526315789473684</v>
       </c>
       <c r="H255" t="n">
-        <v>0.3251964747905731</v>
+        <v>0.3259193003177643</v>
       </c>
     </row>
     <row r="256">
@@ -8117,7 +8117,7 @@
         <v>0.5263157894736842</v>
       </c>
       <c r="H256" t="n">
-        <v>0.01139360014349222</v>
+        <v>0.01347960252314806</v>
       </c>
     </row>
     <row r="257">
@@ -8147,7 +8147,7 @@
         <v>1.184210526315789</v>
       </c>
       <c r="H257" t="n">
-        <v>0.5993899703025818</v>
+        <v>0.6251373291015625</v>
       </c>
     </row>
     <row r="258">
@@ -8177,7 +8177,7 @@
         <v>1.210526315789474</v>
       </c>
       <c r="H258" t="n">
-        <v>0.2886317670345306</v>
+        <v>0.3100955486297607</v>
       </c>
     </row>
     <row r="259">
@@ -8207,7 +8207,7 @@
         <v>0.9210526315789472</v>
       </c>
       <c r="H259" t="n">
-        <v>0.268123596906662</v>
+        <v>0.09787207096815109</v>
       </c>
     </row>
     <row r="260">
@@ -8237,7 +8237,7 @@
         <v>1.921052631578948</v>
       </c>
       <c r="H260" t="n">
-        <v>0.1215487718582153</v>
+        <v>0.1106247827410698</v>
       </c>
     </row>
     <row r="261">
@@ -8267,7 +8267,7 @@
         <v>3.684210526315789</v>
       </c>
       <c r="H261" t="n">
-        <v>0.7447423934936523</v>
+        <v>0.5740684866905212</v>
       </c>
     </row>
     <row r="262">
@@ -8297,7 +8297,7 @@
         <v>1.789473684210526</v>
       </c>
       <c r="H262" t="n">
-        <v>0.1422161757946014</v>
+        <v>0.080058753490448</v>
       </c>
     </row>
     <row r="263">
@@ -8327,7 +8327,7 @@
         <v>3.105263157894737</v>
       </c>
       <c r="H263" t="n">
-        <v>0.6649079918861389</v>
+        <v>0.5624854564666748</v>
       </c>
     </row>
     <row r="264">
@@ -8357,7 +8357,7 @@
         <v>1.342105263157895</v>
       </c>
       <c r="H264" t="n">
-        <v>0.7743573784828186</v>
+        <v>0.6308117508888245</v>
       </c>
     </row>
     <row r="265">
@@ -8387,7 +8387,7 @@
         <v>1.605263157894737</v>
       </c>
       <c r="H265" t="n">
-        <v>0.7050774693489075</v>
+        <v>0.7289354205131531</v>
       </c>
     </row>
     <row r="266">
@@ -8417,7 +8417,7 @@
         <v>2.368421052631579</v>
       </c>
       <c r="H266" t="n">
-        <v>0.5016090273857117</v>
+        <v>0.4124143123626709</v>
       </c>
     </row>
     <row r="267">
@@ -8447,7 +8447,7 @@
         <v>2.210526315789474</v>
       </c>
       <c r="H267" t="n">
-        <v>0.4181956350803375</v>
+        <v>0.1673037558794022</v>
       </c>
     </row>
     <row r="268">
@@ -8477,7 +8477,7 @@
         <v>4.078947368421052</v>
       </c>
       <c r="H268" t="n">
-        <v>0.5915987491607666</v>
+        <v>0.3237490653991699</v>
       </c>
     </row>
     <row r="269">
@@ -8507,7 +8507,7 @@
         <v>1.842105263157895</v>
       </c>
       <c r="H269" t="n">
-        <v>0.5362538695335388</v>
+        <v>0.2977296411991119</v>
       </c>
     </row>
     <row r="270">
@@ -8537,7 +8537,7 @@
         <v>1.131578947368421</v>
       </c>
       <c r="H270" t="n">
-        <v>0.3122722804546356</v>
+        <v>0.2332460433244705</v>
       </c>
     </row>
     <row r="271">
@@ -8567,7 +8567,7 @@
         <v>1.973684210526316</v>
       </c>
       <c r="H271" t="n">
-        <v>0.2523407638072968</v>
+        <v>0.3881802558898926</v>
       </c>
     </row>
     <row r="272">
@@ -8597,7 +8597,7 @@
         <v>0.5</v>
       </c>
       <c r="H272" t="n">
-        <v>0.0743895024061203</v>
+        <v>0.1256227642297745</v>
       </c>
     </row>
     <row r="273">
@@ -8627,7 +8627,7 @@
         <v>1.763157894736842</v>
       </c>
       <c r="H273" t="n">
-        <v>0.1104541197419167</v>
+        <v>0.1410312652587891</v>
       </c>
     </row>
     <row r="274">
@@ -8657,7 +8657,7 @@
         <v>0.8157894736842105</v>
       </c>
       <c r="H274" t="n">
-        <v>0.9407907724380493</v>
+        <v>0.927628755569458</v>
       </c>
     </row>
     <row r="275">
@@ -8687,7 +8687,7 @@
         <v>1.421052631578947</v>
       </c>
       <c r="H275" t="n">
-        <v>0.2196829915046692</v>
+        <v>0.1718585938215256</v>
       </c>
     </row>
     <row r="276">
@@ -8717,7 +8717,7 @@
         <v>2.368421052631579</v>
       </c>
       <c r="H276" t="n">
-        <v>0.130502924323082</v>
+        <v>0.07679214328527451</v>
       </c>
     </row>
     <row r="277">
@@ -8747,7 +8747,7 @@
         <v>2.710526315789474</v>
       </c>
       <c r="H277" t="n">
-        <v>0.3503448367118835</v>
+        <v>0.1937323212623596</v>
       </c>
     </row>
     <row r="278">
@@ -8777,7 +8777,7 @@
         <v>1.868421052631579</v>
       </c>
       <c r="H278" t="n">
-        <v>0.6917358040809631</v>
+        <v>0.6186081171035767</v>
       </c>
     </row>
     <row r="279">
@@ -8807,7 +8807,7 @@
         <v>3.289473684210526</v>
       </c>
       <c r="H279" t="n">
-        <v>0.7624200582504272</v>
+        <v>0.726441502571106</v>
       </c>
     </row>
     <row r="280">
@@ -8837,7 +8837,7 @@
         <v>3.947368421052632</v>
       </c>
       <c r="H280" t="n">
-        <v>0.1474435776472092</v>
+        <v>0.1309333890676498</v>
       </c>
     </row>
     <row r="281">
@@ -11837,7 +11837,7 @@
         <v>0.7368421052631579</v>
       </c>
       <c r="H380" t="n">
-        <v>0.2092773467302322</v>
+        <v>0.3083790242671967</v>
       </c>
     </row>
     <row r="381">
@@ -11867,7 +11867,7 @@
         <v>1.81578947368421</v>
       </c>
       <c r="H381" t="n">
-        <v>0.105974018573761</v>
+        <v>0.08918537944555283</v>
       </c>
     </row>
     <row r="382">
@@ -11897,7 +11897,7 @@
         <v>7.736842105263157</v>
       </c>
       <c r="H382" t="n">
-        <v>0.8854070901870728</v>
+        <v>0.8144672513008118</v>
       </c>
     </row>
     <row r="383">
@@ -11927,7 +11927,7 @@
         <v>2.289473684210526</v>
       </c>
       <c r="H383" t="n">
-        <v>0.7891982793807983</v>
+        <v>0.6404409408569336</v>
       </c>
     </row>
     <row r="384">
@@ -11957,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="H384" t="n">
-        <v>0.8634418845176697</v>
+        <v>0.6810197830200195</v>
       </c>
     </row>
     <row r="385">
@@ -11987,7 +11987,7 @@
         <v>1.526315789473684</v>
       </c>
       <c r="H385" t="n">
-        <v>0.7151197195053101</v>
+        <v>0.6339938044548035</v>
       </c>
     </row>
     <row r="386">
@@ -12017,7 +12017,7 @@
         <v>1.473684210526316</v>
       </c>
       <c r="H386" t="n">
-        <v>0.5142950415611267</v>
+        <v>0.4857182204723358</v>
       </c>
     </row>
     <row r="387">
@@ -12047,7 +12047,7 @@
         <v>2.105263157894737</v>
       </c>
       <c r="H387" t="n">
-        <v>0.7946606874465942</v>
+        <v>0.7670870423316956</v>
       </c>
     </row>
     <row r="388">
@@ -12077,7 +12077,7 @@
         <v>1.263157894736842</v>
       </c>
       <c r="H388" t="n">
-        <v>0.5461243391036987</v>
+        <v>0.6466606259346008</v>
       </c>
     </row>
     <row r="389">
@@ -12107,7 +12107,7 @@
         <v>0.6842105263157895</v>
       </c>
       <c r="H389" t="n">
-        <v>0.6551891565322876</v>
+        <v>0.5870070457458496</v>
       </c>
     </row>
     <row r="390">
@@ -12137,7 +12137,7 @@
         <v>3.473684210526316</v>
       </c>
       <c r="H390" t="n">
-        <v>0.1421398669481277</v>
+        <v>0.05877391993999481</v>
       </c>
     </row>
     <row r="391">
@@ -12167,7 +12167,7 @@
         <v>2.763157894736842</v>
       </c>
       <c r="H391" t="n">
-        <v>0.859071671962738</v>
+        <v>0.8207072615623474</v>
       </c>
     </row>
     <row r="392">
@@ -12197,7 +12197,7 @@
         <v>1.552631578947368</v>
       </c>
       <c r="H392" t="n">
-        <v>0.5229246020317078</v>
+        <v>0.5580012202262878</v>
       </c>
     </row>
     <row r="393">
@@ -12227,7 +12227,7 @@
         <v>1.421052631578947</v>
       </c>
       <c r="H393" t="n">
-        <v>0.2054959237575531</v>
+        <v>0.2259516268968582</v>
       </c>
     </row>
     <row r="394">
@@ -12257,7 +12257,7 @@
         <v>1.947368421052632</v>
       </c>
       <c r="H394" t="n">
-        <v>0.4049542546272278</v>
+        <v>0.590230405330658</v>
       </c>
     </row>
     <row r="395">
@@ -12287,7 +12287,7 @@
         <v>3.5</v>
       </c>
       <c r="H395" t="n">
-        <v>0.5556270480155945</v>
+        <v>0.5286734104156494</v>
       </c>
     </row>
     <row r="396">
@@ -12317,7 +12317,7 @@
         <v>1.263157894736842</v>
       </c>
       <c r="H396" t="n">
-        <v>0.7205791473388672</v>
+        <v>0.8148797750473022</v>
       </c>
     </row>
     <row r="397">
@@ -12347,7 +12347,7 @@
         <v>1.736842105263158</v>
       </c>
       <c r="H397" t="n">
-        <v>0.5309817790985107</v>
+        <v>0.4184781908988953</v>
       </c>
     </row>
     <row r="398">
@@ -12377,7 +12377,7 @@
         <v>1.552631578947368</v>
       </c>
       <c r="H398" t="n">
-        <v>0.7320976853370667</v>
+        <v>0.5107701420783997</v>
       </c>
     </row>
     <row r="399">
@@ -12407,7 +12407,7 @@
         <v>2.052631578947369</v>
       </c>
       <c r="H399" t="n">
-        <v>0.3282296657562256</v>
+        <v>0.6101248860359192</v>
       </c>
     </row>
     <row r="400">
@@ -12437,7 +12437,7 @@
         <v>2.394736842105264</v>
       </c>
       <c r="H400" t="n">
-        <v>0.5490707755088806</v>
+        <v>0.4532009959220886</v>
       </c>
     </row>
     <row r="401">
@@ -12467,7 +12467,7 @@
         <v>1.078947368421053</v>
       </c>
       <c r="H401" t="n">
-        <v>0.1609272211790085</v>
+        <v>0.09097602218389511</v>
       </c>
     </row>
     <row r="402">
@@ -12497,7 +12497,7 @@
         <v>2.289473684210526</v>
       </c>
       <c r="H402" t="n">
-        <v>0.8827316761016846</v>
+        <v>0.9226294755935669</v>
       </c>
     </row>
     <row r="403">
@@ -12527,7 +12527,7 @@
         <v>1.973684210526316</v>
       </c>
       <c r="H403" t="n">
-        <v>0.4847519993782043</v>
+        <v>0.4419349133968353</v>
       </c>
     </row>
     <row r="404">
@@ -12557,7 +12557,7 @@
         <v>8.973684210526315</v>
       </c>
       <c r="H404" t="n">
-        <v>0.8281400203704834</v>
+        <v>0.9283271431922913</v>
       </c>
     </row>
     <row r="405">
@@ -12587,7 +12587,7 @@
         <v>2.210526315789474</v>
       </c>
       <c r="H405" t="n">
-        <v>0.5159497261047363</v>
+        <v>0.705025851726532</v>
       </c>
     </row>
     <row r="406">
@@ -12617,7 +12617,7 @@
         <v>2.605263157894737</v>
       </c>
       <c r="H406" t="n">
-        <v>0.7107741832733154</v>
+        <v>0.4451743364334106</v>
       </c>
     </row>
     <row r="407">
@@ -12647,7 +12647,7 @@
         <v>1.868421052631579</v>
       </c>
       <c r="H407" t="n">
-        <v>0.009127194061875343</v>
+        <v>0.009273452684283257</v>
       </c>
     </row>
     <row r="408">
@@ -12677,7 +12677,7 @@
         <v>3.289473684210526</v>
       </c>
       <c r="H408" t="n">
-        <v>0.06362079083919525</v>
+        <v>0.1769591122865677</v>
       </c>
     </row>
     <row r="409">
@@ -12707,7 +12707,7 @@
         <v>6.447368421052632</v>
       </c>
       <c r="H409" t="n">
-        <v>0.6711001396179199</v>
+        <v>0.6349005103111267</v>
       </c>
     </row>
     <row r="410">
@@ -12737,7 +12737,7 @@
         <v>4.157894736842105</v>
       </c>
       <c r="H410" t="n">
-        <v>0.19443579018116</v>
+        <v>0.1741717904806137</v>
       </c>
     </row>
     <row r="411">
@@ -12767,7 +12767,7 @@
         <v>10.89473684210526</v>
       </c>
       <c r="H411" t="n">
-        <v>0.4724421799182892</v>
+        <v>0.6006166338920593</v>
       </c>
     </row>
     <row r="412">
@@ -12797,7 +12797,7 @@
         <v>8.184210526315789</v>
       </c>
       <c r="H412" t="n">
-        <v>0.4273484349250793</v>
+        <v>0.3354839980602264</v>
       </c>
     </row>
     <row r="413">
@@ -12827,7 +12827,7 @@
         <v>7.578947368421052</v>
       </c>
       <c r="H413" t="n">
-        <v>0.5027584433555603</v>
+        <v>0.5931991934776306</v>
       </c>
     </row>
     <row r="414">
@@ -12857,7 +12857,7 @@
         <v>60.42105263157895</v>
       </c>
       <c r="H414" t="n">
-        <v>0.07730190455913544</v>
+        <v>0.09985040873289108</v>
       </c>
     </row>
     <row r="415">
@@ -12887,7 +12887,7 @@
         <v>17.84210526315789</v>
       </c>
       <c r="H415" t="n">
-        <v>0.9883771538734436</v>
+        <v>0.9898883700370789</v>
       </c>
     </row>
     <row r="416">
@@ -12917,7 +12917,7 @@
         <v>1.894736842105263</v>
       </c>
       <c r="H416" t="n">
-        <v>0.8670269250869751</v>
+        <v>0.6815648078918457</v>
       </c>
     </row>
     <row r="417">
@@ -12947,7 +12947,7 @@
         <v>2.763157894736842</v>
       </c>
       <c r="H417" t="n">
-        <v>0.08037244528532028</v>
+        <v>0.07414965331554413</v>
       </c>
     </row>
     <row r="418">
@@ -12977,7 +12977,7 @@
         <v>3.473684210526316</v>
       </c>
       <c r="H418" t="n">
-        <v>0.1694996654987335</v>
+        <v>0.07153770327568054</v>
       </c>
     </row>
     <row r="419">
@@ -13007,7 +13007,7 @@
         <v>1.026315789473684</v>
       </c>
       <c r="H419" t="n">
-        <v>0.5548650026321411</v>
+        <v>0.4652103185653687</v>
       </c>
     </row>
     <row r="420">
@@ -13037,7 +13037,7 @@
         <v>10.10526315789474</v>
       </c>
       <c r="H420" t="n">
-        <v>0.7893211245536804</v>
+        <v>0.6369408369064331</v>
       </c>
     </row>
     <row r="421">
@@ -13067,7 +13067,7 @@
         <v>29.84210526315789</v>
       </c>
       <c r="H421" t="n">
-        <v>0.6819456219673157</v>
+        <v>0.7633123993873596</v>
       </c>
     </row>
     <row r="422">
@@ -13097,7 +13097,7 @@
         <v>2.394736842105264</v>
       </c>
       <c r="H422" t="n">
-        <v>0.1458725780248642</v>
+        <v>0.09832849353551865</v>
       </c>
     </row>
     <row r="423">
@@ -13127,7 +13127,7 @@
         <v>2.078947368421053</v>
       </c>
       <c r="H423" t="n">
-        <v>0.07757407426834106</v>
+        <v>0.06468958407640457</v>
       </c>
     </row>
     <row r="424">
@@ -13157,7 +13157,7 @@
         <v>2.368421052631579</v>
       </c>
       <c r="H424" t="n">
-        <v>0.08192023634910583</v>
+        <v>0.08821452409029007</v>
       </c>
     </row>
     <row r="425">
@@ -13187,7 +13187,7 @@
         <v>19.07894736842105</v>
       </c>
       <c r="H425" t="n">
-        <v>0.9378700256347656</v>
+        <v>0.9037384390830994</v>
       </c>
     </row>
     <row r="426">
@@ -13217,7 +13217,7 @@
         <v>2.421052631578948</v>
       </c>
       <c r="H426" t="n">
-        <v>0.05136697366833687</v>
+        <v>0.05277317762374878</v>
       </c>
     </row>
     <row r="427">
@@ -13247,7 +13247,7 @@
         <v>2.289473684210526</v>
       </c>
       <c r="H427" t="n">
-        <v>0.4460346698760986</v>
+        <v>0.3334706425666809</v>
       </c>
     </row>
     <row r="428">
@@ -13277,7 +13277,7 @@
         <v>17.15789473684211</v>
       </c>
       <c r="H428" t="n">
-        <v>0.9243873357772827</v>
+        <v>0.9084267616271973</v>
       </c>
     </row>
     <row r="429">
@@ -13307,7 +13307,7 @@
         <v>7.052631578947368</v>
       </c>
       <c r="H429" t="n">
-        <v>0.1986143589019775</v>
+        <v>0.1070387586951256</v>
       </c>
     </row>
     <row r="430">
@@ -13337,7 +13337,7 @@
         <v>7.947368421052632</v>
       </c>
       <c r="H430" t="n">
-        <v>0.9864330887794495</v>
+        <v>0.9570454955101013</v>
       </c>
     </row>
     <row r="431">
@@ -13817,7 +13817,7 @@
         <v>7</v>
       </c>
       <c r="H446" t="n">
-        <v>0.03705465421080589</v>
+        <v>0.04147141799330711</v>
       </c>
     </row>
     <row r="447">
@@ -13847,7 +13847,7 @@
         <v>5</v>
       </c>
       <c r="H447" t="n">
-        <v>0.2233980596065521</v>
+        <v>0.2157171368598938</v>
       </c>
     </row>
     <row r="448">
@@ -13877,7 +13877,7 @@
         <v>6</v>
       </c>
       <c r="H448" t="n">
-        <v>0.1592643409967422</v>
+        <v>0.1355525553226471</v>
       </c>
     </row>
     <row r="449">
@@ -13907,7 +13907,7 @@
         <v>5</v>
       </c>
       <c r="H449" t="n">
-        <v>0.01251301076263189</v>
+        <v>0.0130177941173315</v>
       </c>
     </row>
     <row r="450">
@@ -13937,7 +13937,7 @@
         <v>12</v>
       </c>
       <c r="H450" t="n">
-        <v>0.1785799860954285</v>
+        <v>0.1441562324762344</v>
       </c>
     </row>
     <row r="451">
@@ -13967,7 +13967,7 @@
         <v>22</v>
       </c>
       <c r="H451" t="n">
-        <v>0.1551920026540756</v>
+        <v>0.1865225285291672</v>
       </c>
     </row>
     <row r="452">
@@ -13997,7 +13997,7 @@
         <v>1</v>
       </c>
       <c r="H452" t="n">
-        <v>0.06469999998807907</v>
+        <v>0.08028609305620193</v>
       </c>
     </row>
     <row r="453">
@@ -14027,7 +14027,7 @@
         <v>2</v>
       </c>
       <c r="H453" t="n">
-        <v>0.09704478085041046</v>
+        <v>0.08483521640300751</v>
       </c>
     </row>
     <row r="454">
@@ -14057,7 +14057,7 @@
         <v>23</v>
       </c>
       <c r="H454" t="n">
-        <v>0.3681038916110992</v>
+        <v>0.3656766712665558</v>
       </c>
     </row>
     <row r="455">
@@ -14087,7 +14087,7 @@
         <v>8</v>
       </c>
       <c r="H455" t="n">
-        <v>0.0141674904152751</v>
+        <v>0.01141714956611395</v>
       </c>
     </row>
     <row r="456">
@@ -14117,7 +14117,7 @@
         <v>1</v>
       </c>
       <c r="H456" t="n">
-        <v>0.1550752073526382</v>
+        <v>0.1397836953401566</v>
       </c>
     </row>
     <row r="457">
@@ -14147,7 +14147,7 @@
         <v>6</v>
       </c>
       <c r="H457" t="n">
-        <v>0.008669102564454079</v>
+        <v>0.009608794935047626</v>
       </c>
     </row>
     <row r="458">
@@ -14177,7 +14177,7 @@
         <v>8</v>
       </c>
       <c r="H458" t="n">
-        <v>0.08744934946298599</v>
+        <v>0.09502976387739182</v>
       </c>
     </row>
     <row r="459">
@@ -14207,7 +14207,7 @@
         <v>17</v>
       </c>
       <c r="H459" t="n">
-        <v>0.1383670419454575</v>
+        <v>0.1579186767339706</v>
       </c>
     </row>
     <row r="460">
@@ -14237,7 +14237,7 @@
         <v>8</v>
       </c>
       <c r="H460" t="n">
-        <v>0.02585469931364059</v>
+        <v>0.02677479945123196</v>
       </c>
     </row>
     <row r="461">
@@ -14267,7 +14267,7 @@
         <v>8</v>
       </c>
       <c r="H461" t="n">
-        <v>0.7087998390197754</v>
+        <v>0.6910462379455566</v>
       </c>
     </row>
     <row r="462">
@@ -14297,7 +14297,7 @@
         <v>0</v>
       </c>
       <c r="H462" t="n">
-        <v>0.03194620832800865</v>
+        <v>0.02901884168386459</v>
       </c>
     </row>
     <row r="463">
@@ -14327,7 +14327,7 @@
         <v>5</v>
       </c>
       <c r="H463" t="n">
-        <v>0.05702482908964157</v>
+        <v>0.0569169893860817</v>
       </c>
     </row>
     <row r="464">
@@ -14357,7 +14357,7 @@
         <v>59</v>
       </c>
       <c r="H464" t="n">
-        <v>0.3983010053634644</v>
+        <v>0.4617931842803955</v>
       </c>
     </row>
     <row r="465">
@@ -14387,7 +14387,7 @@
         <v>12</v>
       </c>
       <c r="H465" t="n">
-        <v>0.1184881702065468</v>
+        <v>0.1656229496002197</v>
       </c>
     </row>
     <row r="466">
@@ -14417,7 +14417,7 @@
         <v>8</v>
       </c>
       <c r="H466" t="n">
-        <v>0.01924802735447884</v>
+        <v>0.01879030279815197</v>
       </c>
     </row>
     <row r="467">
@@ -14447,7 +14447,7 @@
         <v>14</v>
       </c>
       <c r="H467" t="n">
-        <v>0.6936126947402954</v>
+        <v>0.729267954826355</v>
       </c>
     </row>
     <row r="468">
@@ -14477,7 +14477,7 @@
         <v>9</v>
       </c>
       <c r="H468" t="n">
-        <v>0.4514763653278351</v>
+        <v>0.5013312101364136</v>
       </c>
     </row>
     <row r="469">
@@ -14507,7 +14507,7 @@
         <v>8</v>
       </c>
       <c r="H469" t="n">
-        <v>0.0605330765247345</v>
+        <v>0.06550627946853638</v>
       </c>
     </row>
     <row r="470">
@@ -14537,7 +14537,7 @@
         <v>5</v>
       </c>
       <c r="H470" t="n">
-        <v>0.3596931397914886</v>
+        <v>0.35758176445961</v>
       </c>
     </row>
     <row r="471">
@@ -14567,7 +14567,7 @@
         <v>8</v>
       </c>
       <c r="H471" t="n">
-        <v>0.03057688288390636</v>
+        <v>0.03052503243088722</v>
       </c>
     </row>
     <row r="472">
@@ -14597,7 +14597,7 @@
         <v>7</v>
       </c>
       <c r="H472" t="n">
-        <v>0.02391777187585831</v>
+        <v>0.01449166424572468</v>
       </c>
     </row>
     <row r="473">
@@ -14627,7 +14627,7 @@
         <v>5</v>
       </c>
       <c r="H473" t="n">
-        <v>0.03530758246779442</v>
+        <v>0.0437810942530632</v>
       </c>
     </row>
     <row r="474">
@@ -14657,7 +14657,7 @@
         <v>4</v>
       </c>
       <c r="H474" t="n">
-        <v>0.0578574426472187</v>
+        <v>0.0376867838203907</v>
       </c>
     </row>
     <row r="475">
@@ -14687,7 +14687,7 @@
         <v>8</v>
       </c>
       <c r="H475" t="n">
-        <v>0.8602404594421387</v>
+        <v>0.8333587050437927</v>
       </c>
     </row>
     <row r="476">
@@ -14717,7 +14717,7 @@
         <v>8</v>
       </c>
       <c r="H476" t="n">
-        <v>0.106442466378212</v>
+        <v>0.07811141759157181</v>
       </c>
     </row>
     <row r="477">
@@ -14747,7 +14747,7 @@
         <v>13</v>
       </c>
       <c r="H477" t="n">
-        <v>0.4703585207462311</v>
+        <v>0.4311246573925018</v>
       </c>
     </row>
     <row r="478">
@@ -14777,7 +14777,7 @@
         <v>7</v>
       </c>
       <c r="H478" t="n">
-        <v>0.363030731678009</v>
+        <v>0.2195664644241333</v>
       </c>
     </row>
     <row r="479">
@@ -14807,7 +14807,7 @@
         <v>12</v>
       </c>
       <c r="H479" t="n">
-        <v>0.5924601554870605</v>
+        <v>0.5946973562240601</v>
       </c>
     </row>
     <row r="480">
@@ -14837,7 +14837,7 @@
         <v>10</v>
       </c>
       <c r="H480" t="n">
-        <v>0.4034859240055084</v>
+        <v>0.3327632248401642</v>
       </c>
     </row>
     <row r="481">
@@ -14867,7 +14867,7 @@
         <v>8</v>
       </c>
       <c r="H481" t="n">
-        <v>0.1331523805856705</v>
+        <v>0.1285273283720016</v>
       </c>
     </row>
     <row r="482">
@@ -14897,7 +14897,7 @@
         <v>8</v>
       </c>
       <c r="H482" t="n">
-        <v>0.3577269315719604</v>
+        <v>0.2727998793125153</v>
       </c>
     </row>
     <row r="483">
@@ -14927,7 +14927,7 @@
         <v>14</v>
       </c>
       <c r="H483" t="n">
-        <v>0.8157445788383484</v>
+        <v>0.7635380029678345</v>
       </c>
     </row>
     <row r="484">
@@ -14957,7 +14957,7 @@
         <v>7</v>
       </c>
       <c r="H484" t="n">
-        <v>0.003212037030607462</v>
+        <v>0.004131481517106295</v>
       </c>
     </row>
     <row r="485">
@@ -14987,7 +14987,7 @@
         <v>19</v>
       </c>
       <c r="H485" t="n">
-        <v>0.5885618329048157</v>
+        <v>0.7183759212493896</v>
       </c>
     </row>
     <row r="486">
@@ -15017,7 +15017,7 @@
         <v>8</v>
       </c>
       <c r="H486" t="n">
-        <v>0.2271794825792313</v>
+        <v>0.2256078273057938</v>
       </c>
     </row>
     <row r="487">
@@ -15047,7 +15047,7 @@
         <v>10</v>
       </c>
       <c r="H487" t="n">
-        <v>0.4553369581699371</v>
+        <v>0.4057459533214569</v>
       </c>
     </row>
     <row r="488">
@@ -15077,7 +15077,7 @@
         <v>3</v>
       </c>
       <c r="H488" t="n">
-        <v>0.05038722977042198</v>
+        <v>0.05713355541229248</v>
       </c>
     </row>
     <row r="489">
@@ -15107,7 +15107,7 @@
         <v>10</v>
       </c>
       <c r="H489" t="n">
-        <v>0.206858366727829</v>
+        <v>0.1794942766427994</v>
       </c>
     </row>
     <row r="490">
@@ -15137,7 +15137,7 @@
         <v>8</v>
       </c>
       <c r="H490" t="n">
-        <v>0.1742022782564163</v>
+        <v>0.121984988451004</v>
       </c>
     </row>
     <row r="491">
@@ -15167,7 +15167,7 @@
         <v>8</v>
       </c>
       <c r="H491" t="n">
-        <v>0.07888826727867126</v>
+        <v>0.06646739691495895</v>
       </c>
     </row>
     <row r="492">
@@ -15197,7 +15197,7 @@
         <v>26</v>
       </c>
       <c r="H492" t="n">
-        <v>0.3205793499946594</v>
+        <v>0.2712293863296509</v>
       </c>
     </row>
     <row r="493">
@@ -15227,7 +15227,7 @@
         <v>62</v>
       </c>
       <c r="H493" t="n">
-        <v>0.3076061010360718</v>
+        <v>0.3122449815273285</v>
       </c>
     </row>
     <row r="494">
@@ -15257,7 +15257,7 @@
         <v>8</v>
       </c>
       <c r="H494" t="n">
-        <v>0.2417204976081848</v>
+        <v>0.2436235249042511</v>
       </c>
     </row>
     <row r="495">
@@ -15287,7 +15287,7 @@
         <v>8</v>
       </c>
       <c r="H495" t="n">
-        <v>0.02088277414441109</v>
+        <v>0.03067917004227638</v>
       </c>
     </row>
     <row r="496">
@@ -15317,7 +15317,7 @@
         <v>8</v>
       </c>
       <c r="H496" t="n">
-        <v>0.04540746659040451</v>
+        <v>0.03713294863700867</v>
       </c>
     </row>
     <row r="497">
@@ -15347,7 +15347,7 @@
         <v>19</v>
       </c>
       <c r="H497" t="n">
-        <v>0.1488006412982941</v>
+        <v>0.1563738733530045</v>
       </c>
     </row>
     <row r="498">
@@ -15377,7 +15377,7 @@
         <v>2</v>
       </c>
       <c r="H498" t="n">
-        <v>0.03339338675141335</v>
+        <v>0.03356439247727394</v>
       </c>
     </row>
     <row r="499">
@@ -15407,7 +15407,7 @@
         <v>8</v>
       </c>
       <c r="H499" t="n">
-        <v>0.2840295732021332</v>
+        <v>0.3402070701122284</v>
       </c>
     </row>
     <row r="500">
@@ -15437,7 +15437,7 @@
         <v>6</v>
       </c>
       <c r="H500" t="n">
-        <v>0.1314427554607391</v>
+        <v>0.09213894605636597</v>
       </c>
     </row>
     <row r="501">
@@ -15467,7 +15467,7 @@
         <v>7</v>
       </c>
       <c r="H501" t="n">
-        <v>0.04510098695755005</v>
+        <v>0.02694662846624851</v>
       </c>
     </row>
     <row r="502">
@@ -15497,7 +15497,7 @@
         <v>2</v>
       </c>
       <c r="H502" t="n">
-        <v>0.1384830921888351</v>
+        <v>0.1289477050304413</v>
       </c>
     </row>
     <row r="503">
@@ -15527,7 +15527,7 @@
         <v>8</v>
       </c>
       <c r="H503" t="n">
-        <v>0.01105101313441992</v>
+        <v>0.009227151982486248</v>
       </c>
     </row>
     <row r="504">
@@ -15557,7 +15557,7 @@
         <v>8</v>
       </c>
       <c r="H504" t="n">
-        <v>0.02932370454072952</v>
+        <v>0.02320079691708088</v>
       </c>
     </row>
     <row r="505">
@@ -15587,7 +15587,7 @@
         <v>1.657894736842105</v>
       </c>
       <c r="H505" t="n">
-        <v>0.4449006915092468</v>
+        <v>0.2600487470626831</v>
       </c>
     </row>
     <row r="506">
@@ -15617,7 +15617,7 @@
         <v>0.8157894736842105</v>
       </c>
       <c r="H506" t="n">
-        <v>0.4169493913650513</v>
+        <v>0.6134600043296814</v>
       </c>
     </row>
     <row r="507">
@@ -15647,7 +15647,7 @@
         <v>0.8947368421052632</v>
       </c>
       <c r="H507" t="n">
-        <v>0.866754949092865</v>
+        <v>0.8505183458328247</v>
       </c>
     </row>
     <row r="508">
@@ -15677,7 +15677,7 @@
         <v>2</v>
       </c>
       <c r="H508" t="n">
-        <v>0.6813837289810181</v>
+        <v>0.7663690447807312</v>
       </c>
     </row>
     <row r="509">
@@ -15707,7 +15707,7 @@
         <v>1.763157894736842</v>
       </c>
       <c r="H509" t="n">
-        <v>0.411393404006958</v>
+        <v>0.3417277932167053</v>
       </c>
     </row>
     <row r="510">
@@ -15737,7 +15737,7 @@
         <v>1.81578947368421</v>
       </c>
       <c r="H510" t="n">
-        <v>0.7347530126571655</v>
+        <v>0.694827139377594</v>
       </c>
     </row>
     <row r="511">
@@ -15767,7 +15767,7 @@
         <v>1.236842105263158</v>
       </c>
       <c r="H511" t="n">
-        <v>0.8670892119407654</v>
+        <v>0.8716325163841248</v>
       </c>
     </row>
     <row r="512">
@@ -15797,7 +15797,7 @@
         <v>1.210526315789474</v>
       </c>
       <c r="H512" t="n">
-        <v>0.07697582244873047</v>
+        <v>0.1002442985773087</v>
       </c>
     </row>
     <row r="513">
@@ -15827,7 +15827,7 @@
         <v>1.421052631578947</v>
       </c>
       <c r="H513" t="n">
-        <v>0.6128880381584167</v>
+        <v>0.5323945879936218</v>
       </c>
     </row>
     <row r="514">
@@ -15857,7 +15857,7 @@
         <v>2.710526315789474</v>
       </c>
       <c r="H514" t="n">
-        <v>0.7592893838882446</v>
+        <v>0.808262050151825</v>
       </c>
     </row>
     <row r="515">
@@ -15887,7 +15887,7 @@
         <v>0.7631578947368421</v>
       </c>
       <c r="H515" t="n">
-        <v>0.2816107571125031</v>
+        <v>0.3994359076023102</v>
       </c>
     </row>
     <row r="516">
@@ -15917,7 +15917,7 @@
         <v>3.447368421052631</v>
       </c>
       <c r="H516" t="n">
-        <v>0.139082208275795</v>
+        <v>0.450908899307251</v>
       </c>
     </row>
     <row r="517">
@@ -15947,7 +15947,7 @@
         <v>0.5</v>
       </c>
       <c r="H517" t="n">
-        <v>0.8124314546585083</v>
+        <v>0.5469902157783508</v>
       </c>
     </row>
     <row r="518">
@@ -15977,7 +15977,7 @@
         <v>1.842105263157895</v>
       </c>
       <c r="H518" t="n">
-        <v>0.369904488325119</v>
+        <v>0.4208725690841675</v>
       </c>
     </row>
     <row r="519">
@@ -16007,7 +16007,7 @@
         <v>1.473684210526316</v>
       </c>
       <c r="H519" t="n">
-        <v>0.6632565855979919</v>
+        <v>0.7254534959793091</v>
       </c>
     </row>
     <row r="520">
@@ -16037,7 +16037,7 @@
         <v>2.473684210526316</v>
       </c>
       <c r="H520" t="n">
-        <v>0.8897421360015869</v>
+        <v>0.8510774374008179</v>
       </c>
     </row>
     <row r="521">
@@ -16067,7 +16067,7 @@
         <v>2.157894736842105</v>
       </c>
       <c r="H521" t="n">
-        <v>0.786969006061554</v>
+        <v>0.7214821577072144</v>
       </c>
     </row>
     <row r="522">
@@ -16097,7 +16097,7 @@
         <v>1</v>
       </c>
       <c r="H522" t="n">
-        <v>0.4837128221988678</v>
+        <v>0.6332964897155762</v>
       </c>
     </row>
     <row r="523">
@@ -16127,7 +16127,7 @@
         <v>1.289473684210526</v>
       </c>
       <c r="H523" t="n">
-        <v>0.4007644653320312</v>
+        <v>0.3098936676979065</v>
       </c>
     </row>
     <row r="524">
@@ -16157,7 +16157,7 @@
         <v>4.5</v>
       </c>
       <c r="H524" t="n">
-        <v>0.7092671990394592</v>
+        <v>0.6956372857093811</v>
       </c>
     </row>
     <row r="525">
@@ -16187,7 +16187,7 @@
         <v>1.421052631578947</v>
       </c>
       <c r="H525" t="n">
-        <v>0.7644495368003845</v>
+        <v>0.6918196678161621</v>
       </c>
     </row>
     <row r="526">
@@ -16217,7 +16217,7 @@
         <v>6.763157894736842</v>
       </c>
       <c r="H526" t="n">
-        <v>0.7493036389350891</v>
+        <v>0.7175782918930054</v>
       </c>
     </row>
     <row r="527">
@@ -16247,7 +16247,7 @@
         <v>4.763157894736842</v>
       </c>
       <c r="H527" t="n">
-        <v>0.5595888495445251</v>
+        <v>0.3634811341762543</v>
       </c>
     </row>
     <row r="528">
@@ -16277,7 +16277,7 @@
         <v>1.868421052631579</v>
       </c>
       <c r="H528" t="n">
-        <v>0.8305983543395996</v>
+        <v>0.7692746520042419</v>
       </c>
     </row>
     <row r="529">
@@ -16307,7 +16307,7 @@
         <v>1.157894736842105</v>
       </c>
       <c r="H529" t="n">
-        <v>0.1930621415376663</v>
+        <v>0.3115558326244354</v>
       </c>
     </row>
     <row r="530">
@@ -16337,7 +16337,7 @@
         <v>2.631578947368421</v>
       </c>
       <c r="H530" t="n">
-        <v>0.6071646809577942</v>
+        <v>0.6479353904724121</v>
       </c>
     </row>
     <row r="531">
@@ -16367,7 +16367,7 @@
         <v>2.289473684210526</v>
       </c>
       <c r="H531" t="n">
-        <v>0.3574273884296417</v>
+        <v>0.3395239114761353</v>
       </c>
     </row>
     <row r="532">
@@ -16397,7 +16397,7 @@
         <v>3.315789473684211</v>
       </c>
       <c r="H532" t="n">
-        <v>0.9154215455055237</v>
+        <v>0.9283303022384644</v>
       </c>
     </row>
     <row r="533">
@@ -16427,7 +16427,7 @@
         <v>4.526315789473684</v>
       </c>
       <c r="H533" t="n">
-        <v>0.03861522302031517</v>
+        <v>0.04713773354887962</v>
       </c>
     </row>
     <row r="534">
@@ -16457,7 +16457,7 @@
         <v>0.8947368421052632</v>
       </c>
       <c r="H534" t="n">
-        <v>0.7692049145698547</v>
+        <v>0.8657248616218567</v>
       </c>
     </row>
     <row r="535">
@@ -16487,7 +16487,7 @@
         <v>1.5</v>
       </c>
       <c r="H535" t="n">
-        <v>0.9019309282302856</v>
+        <v>0.9458020925521851</v>
       </c>
     </row>
     <row r="536">
@@ -16517,7 +16517,7 @@
         <v>7.394736842105263</v>
       </c>
       <c r="H536" t="n">
-        <v>0.3754426836967468</v>
+        <v>0.2782392203807831</v>
       </c>
     </row>
     <row r="537">
@@ -16547,7 +16547,7 @@
         <v>16.57894736842105</v>
       </c>
       <c r="H537" t="n">
-        <v>0.994658887386322</v>
+        <v>0.9928144812583923</v>
       </c>
     </row>
     <row r="538">
@@ -16577,7 +16577,7 @@
         <v>10.21052631578947</v>
       </c>
       <c r="H538" t="n">
-        <v>0.9830180406570435</v>
+        <v>0.9864050149917603</v>
       </c>
     </row>
     <row r="539">
@@ -16607,7 +16607,7 @@
         <v>22.63157894736842</v>
       </c>
       <c r="H539" t="n">
-        <v>0.9295961856842041</v>
+        <v>0.9307107925415039</v>
       </c>
     </row>
     <row r="540">
@@ -16637,7 +16637,7 @@
         <v>8.789473684210526</v>
       </c>
       <c r="H540" t="n">
-        <v>0.8665473461151123</v>
+        <v>0.7788892984390259</v>
       </c>
     </row>
     <row r="541">
@@ -16667,7 +16667,7 @@
         <v>9.868421052631581</v>
       </c>
       <c r="H541" t="n">
-        <v>0.06888400763273239</v>
+        <v>0.1955353319644928</v>
       </c>
     </row>
     <row r="542">
@@ -16697,7 +16697,7 @@
         <v>1.210526315789474</v>
       </c>
       <c r="H542" t="n">
-        <v>0.03075857274234295</v>
+        <v>0.0760892927646637</v>
       </c>
     </row>
     <row r="543">
@@ -16727,7 +16727,7 @@
         <v>16.86842105263158</v>
       </c>
       <c r="H543" t="n">
-        <v>0.622998058795929</v>
+        <v>0.5669634938240051</v>
       </c>
     </row>
     <row r="544">
@@ -16757,7 +16757,7 @@
         <v>1.473684210526316</v>
       </c>
       <c r="H544" t="n">
-        <v>0.2020173072814941</v>
+        <v>0.1644924432039261</v>
       </c>
     </row>
     <row r="545">
@@ -16787,7 +16787,7 @@
         <v>12.57894736842105</v>
       </c>
       <c r="H545" t="n">
-        <v>0.3541211783885956</v>
+        <v>0.3309343159198761</v>
       </c>
     </row>
     <row r="546">
@@ -16817,7 +16817,7 @@
         <v>8.605263157894736</v>
       </c>
       <c r="H546" t="n">
-        <v>0.9693677425384521</v>
+        <v>0.9748243093490601</v>
       </c>
     </row>
     <row r="547">
@@ -16847,7 +16847,7 @@
         <v>0.5789473684210527</v>
       </c>
       <c r="H547" t="n">
-        <v>0.05781110748648643</v>
+        <v>0.07515880465507507</v>
       </c>
     </row>
     <row r="548">
@@ -16877,7 +16877,7 @@
         <v>45.63157894736842</v>
       </c>
       <c r="H548" t="n">
-        <v>0.30118128657341</v>
+        <v>0.1477426290512085</v>
       </c>
     </row>
     <row r="549">
@@ -16907,7 +16907,7 @@
         <v>10.36842105263158</v>
       </c>
       <c r="H549" t="n">
-        <v>0.8476280570030212</v>
+        <v>0.843237042427063</v>
       </c>
     </row>
     <row r="550">
@@ -16937,7 +16937,7 @@
         <v>1.052631578947368</v>
       </c>
       <c r="H550" t="n">
-        <v>0.9780114889144897</v>
+        <v>0.9726430773735046</v>
       </c>
     </row>
     <row r="551">
@@ -16967,7 +16967,7 @@
         <v>1.131578947368421</v>
       </c>
       <c r="H551" t="n">
-        <v>0.4246167540550232</v>
+        <v>0.4465589821338654</v>
       </c>
     </row>
     <row r="552">
@@ -16997,7 +16997,7 @@
         <v>5.105263157894737</v>
       </c>
       <c r="H552" t="n">
-        <v>0.215761125087738</v>
+        <v>0.2387400716543198</v>
       </c>
     </row>
     <row r="553">
@@ -17027,7 +17027,7 @@
         <v>38.86842105263158</v>
       </c>
       <c r="H553" t="n">
-        <v>0.3587696850299835</v>
+        <v>0.341198205947876</v>
       </c>
     </row>
     <row r="554">
@@ -17057,7 +17057,7 @@
         <v>5.105263157894737</v>
       </c>
       <c r="H554" t="n">
-        <v>0.03096979297697544</v>
+        <v>0.05862745270133018</v>
       </c>
     </row>
     <row r="555">
@@ -17087,7 +17087,7 @@
         <v>23.92105263157895</v>
       </c>
       <c r="H555" t="n">
-        <v>0.9647639393806458</v>
+        <v>0.9792417883872986</v>
       </c>
     </row>
     <row r="556">
@@ -17567,7 +17567,7 @@
         <v>44</v>
       </c>
       <c r="H571" t="n">
-        <v>0.7862328886985779</v>
+        <v>0.8180338740348816</v>
       </c>
     </row>
     <row r="572">
@@ -17597,7 +17597,7 @@
         <v>6</v>
       </c>
       <c r="H572" t="n">
-        <v>0.08593765646219254</v>
+        <v>0.1223030537366867</v>
       </c>
     </row>
     <row r="573">
@@ -17627,7 +17627,7 @@
         <v>8</v>
       </c>
       <c r="H573" t="n">
-        <v>0.003380682552233338</v>
+        <v>0.00590251199901104</v>
       </c>
     </row>
     <row r="574">
@@ -17657,7 +17657,7 @@
         <v>32</v>
       </c>
       <c r="H574" t="n">
-        <v>0.8231367468833923</v>
+        <v>0.5213993787765503</v>
       </c>
     </row>
     <row r="575">
@@ -17687,7 +17687,7 @@
         <v>15</v>
       </c>
       <c r="H575" t="n">
-        <v>0.09596249461174011</v>
+        <v>0.06072880700230598</v>
       </c>
     </row>
     <row r="576">
@@ -17717,7 +17717,7 @@
         <v>8</v>
       </c>
       <c r="H576" t="n">
-        <v>0.02977132983505726</v>
+        <v>0.04823929816484451</v>
       </c>
     </row>
     <row r="577">
@@ -17747,7 +17747,7 @@
         <v>18</v>
       </c>
       <c r="H577" t="n">
-        <v>0.8261911869049072</v>
+        <v>0.7864096164703369</v>
       </c>
     </row>
     <row r="578">
@@ -17777,7 +17777,7 @@
         <v>7</v>
       </c>
       <c r="H578" t="n">
-        <v>0.1348688453435898</v>
+        <v>0.1611915528774261</v>
       </c>
     </row>
     <row r="579">
@@ -17807,7 +17807,7 @@
         <v>13</v>
       </c>
       <c r="H579" t="n">
-        <v>0.2779399454593658</v>
+        <v>0.162043109536171</v>
       </c>
     </row>
     <row r="580">
@@ -17837,7 +17837,7 @@
         <v>7</v>
       </c>
       <c r="H580" t="n">
-        <v>0.1053812205791473</v>
+        <v>0.09269118309020996</v>
       </c>
     </row>
     <row r="581">
@@ -17867,7 +17867,7 @@
         <v>5</v>
       </c>
       <c r="H581" t="n">
-        <v>0.2310449928045273</v>
+        <v>0.2266016453504562</v>
       </c>
     </row>
     <row r="582">
@@ -17897,7 +17897,7 @@
         <v>18</v>
       </c>
       <c r="H582" t="n">
-        <v>0.1226557567715645</v>
+        <v>0.3881699740886688</v>
       </c>
     </row>
     <row r="583">
@@ -17927,7 +17927,7 @@
         <v>8</v>
       </c>
       <c r="H583" t="n">
-        <v>0.008225428871810436</v>
+        <v>0.004330192226916552</v>
       </c>
     </row>
     <row r="584">
@@ -17957,7 +17957,7 @@
         <v>44</v>
       </c>
       <c r="H584" t="n">
-        <v>0.8635401725769043</v>
+        <v>0.7943805456161499</v>
       </c>
     </row>
     <row r="585">
@@ -17987,7 +17987,7 @@
         <v>11</v>
       </c>
       <c r="H585" t="n">
-        <v>0.7947641015052795</v>
+        <v>0.7569905519485474</v>
       </c>
     </row>
     <row r="586">
@@ -18017,7 +18017,7 @@
         <v>12</v>
       </c>
       <c r="H586" t="n">
-        <v>0.2730571925640106</v>
+        <v>0.166469931602478</v>
       </c>
     </row>
     <row r="587">
@@ -18047,7 +18047,7 @@
         <v>5</v>
       </c>
       <c r="H587" t="n">
-        <v>0.02505189180374146</v>
+        <v>0.02184637077152729</v>
       </c>
     </row>
     <row r="588">
@@ -18077,7 +18077,7 @@
         <v>8</v>
       </c>
       <c r="H588" t="n">
-        <v>0.08166010677814484</v>
+        <v>0.08287162333726883</v>
       </c>
     </row>
     <row r="589">
@@ -18107,7 +18107,7 @@
         <v>13</v>
       </c>
       <c r="H589" t="n">
-        <v>0.4418723881244659</v>
+        <v>0.5223585963249207</v>
       </c>
     </row>
     <row r="590">
@@ -18137,7 +18137,7 @@
         <v>4</v>
       </c>
       <c r="H590" t="n">
-        <v>0.0138798113912344</v>
+        <v>0.01295087859034538</v>
       </c>
     </row>
     <row r="591">
@@ -18167,7 +18167,7 @@
         <v>5</v>
       </c>
       <c r="H591" t="n">
-        <v>0.1829410493373871</v>
+        <v>0.1235383227467537</v>
       </c>
     </row>
     <row r="592">
@@ -18197,7 +18197,7 @@
         <v>32</v>
       </c>
       <c r="H592" t="n">
-        <v>0.305363655090332</v>
+        <v>0.3841775059700012</v>
       </c>
     </row>
     <row r="593">
@@ -18227,7 +18227,7 @@
         <v>11</v>
       </c>
       <c r="H593" t="n">
-        <v>0.05041330680251122</v>
+        <v>0.05321422219276428</v>
       </c>
     </row>
     <row r="594">
@@ -18257,7 +18257,7 @@
         <v>13</v>
       </c>
       <c r="H594" t="n">
-        <v>0.6384140253067017</v>
+        <v>0.6928066611289978</v>
       </c>
     </row>
     <row r="595">
@@ -18287,7 +18287,7 @@
         <v>27</v>
       </c>
       <c r="H595" t="n">
-        <v>0.8565430045127869</v>
+        <v>0.7007895708084106</v>
       </c>
     </row>
     <row r="596">
@@ -18317,7 +18317,7 @@
         <v>14</v>
       </c>
       <c r="H596" t="n">
-        <v>0.2201785743236542</v>
+        <v>0.2454008460044861</v>
       </c>
     </row>
     <row r="597">
@@ -18347,7 +18347,7 @@
         <v>8</v>
       </c>
       <c r="H597" t="n">
-        <v>0.01161959674209356</v>
+        <v>0.02414598502218723</v>
       </c>
     </row>
     <row r="598">
@@ -18377,7 +18377,7 @@
         <v>1</v>
       </c>
       <c r="H598" t="n">
-        <v>0.07305624336004257</v>
+        <v>0.0539458841085434</v>
       </c>
     </row>
     <row r="599">
@@ -18407,7 +18407,7 @@
         <v>21</v>
       </c>
       <c r="H599" t="n">
-        <v>0.3507205247879028</v>
+        <v>0.3591208755970001</v>
       </c>
     </row>
     <row r="600">
@@ -18437,7 +18437,7 @@
         <v>8</v>
       </c>
       <c r="H600" t="n">
-        <v>0.01348643284291029</v>
+        <v>0.008477143943309784</v>
       </c>
     </row>
     <row r="601">
@@ -18467,7 +18467,7 @@
         <v>11</v>
       </c>
       <c r="H601" t="n">
-        <v>0.01002882700413465</v>
+        <v>0.004165193531662226</v>
       </c>
     </row>
     <row r="602">
@@ -18497,7 +18497,7 @@
         <v>5</v>
       </c>
       <c r="H602" t="n">
-        <v>0.05032556504011154</v>
+        <v>0.02764454670250416</v>
       </c>
     </row>
     <row r="603">
@@ -18527,7 +18527,7 @@
         <v>8</v>
       </c>
       <c r="H603" t="n">
-        <v>0.1062494814395905</v>
+        <v>0.06315069645643234</v>
       </c>
     </row>
     <row r="604">
@@ -18557,7 +18557,7 @@
         <v>5</v>
       </c>
       <c r="H604" t="n">
-        <v>0.02447878755629063</v>
+        <v>0.02438165619969368</v>
       </c>
     </row>
     <row r="605">
@@ -18587,7 +18587,7 @@
         <v>6</v>
       </c>
       <c r="H605" t="n">
-        <v>0.1025584116578102</v>
+        <v>0.1107639819383621</v>
       </c>
     </row>
     <row r="606">
@@ -18617,7 +18617,7 @@
         <v>8</v>
       </c>
       <c r="H606" t="n">
-        <v>0.200664684176445</v>
+        <v>0.1109438017010689</v>
       </c>
     </row>
     <row r="607">
@@ -18647,7 +18647,7 @@
         <v>8</v>
       </c>
       <c r="H607" t="n">
-        <v>0.399253636598587</v>
+        <v>0.4706315398216248</v>
       </c>
     </row>
     <row r="608">
@@ -18677,7 +18677,7 @@
         <v>3</v>
       </c>
       <c r="H608" t="n">
-        <v>0.007438997738063335</v>
+        <v>0.01267537660896778</v>
       </c>
     </row>
     <row r="609">
@@ -18707,7 +18707,7 @@
         <v>8</v>
       </c>
       <c r="H609" t="n">
-        <v>0.07168465852737427</v>
+        <v>0.08010037243366241</v>
       </c>
     </row>
     <row r="610">
@@ -18737,7 +18737,7 @@
         <v>8</v>
       </c>
       <c r="H610" t="n">
-        <v>0.137351393699646</v>
+        <v>0.2111094892024994</v>
       </c>
     </row>
     <row r="611">
@@ -18767,7 +18767,7 @@
         <v>4</v>
       </c>
       <c r="H611" t="n">
-        <v>0.152823731303215</v>
+        <v>0.1097418963909149</v>
       </c>
     </row>
     <row r="612">
@@ -18797,7 +18797,7 @@
         <v>8</v>
       </c>
       <c r="H612" t="n">
-        <v>0.01266230829060078</v>
+        <v>0.0225487295538187</v>
       </c>
     </row>
     <row r="613">
@@ -18827,7 +18827,7 @@
         <v>5</v>
       </c>
       <c r="H613" t="n">
-        <v>0.06310845911502838</v>
+        <v>0.05156504362821579</v>
       </c>
     </row>
     <row r="614">
@@ -18857,7 +18857,7 @@
         <v>16</v>
       </c>
       <c r="H614" t="n">
-        <v>0.3780232667922974</v>
+        <v>0.3628620207309723</v>
       </c>
     </row>
     <row r="615">
@@ -18887,7 +18887,7 @@
         <v>20</v>
       </c>
       <c r="H615" t="n">
-        <v>0.6571322679519653</v>
+        <v>0.8304014205932617</v>
       </c>
     </row>
     <row r="616">
@@ -18917,7 +18917,7 @@
         <v>6</v>
       </c>
       <c r="H616" t="n">
-        <v>0.02562194876372814</v>
+        <v>0.03891678899526596</v>
       </c>
     </row>
     <row r="617">
@@ -18947,7 +18947,7 @@
         <v>3</v>
       </c>
       <c r="H617" t="n">
-        <v>0.005862458143383265</v>
+        <v>0.00654577324166894</v>
       </c>
     </row>
     <row r="618">
@@ -18977,7 +18977,7 @@
         <v>5</v>
       </c>
       <c r="H618" t="n">
-        <v>0.01134146936237812</v>
+        <v>0.005662667565047741</v>
       </c>
     </row>
     <row r="619">
@@ -19007,7 +19007,7 @@
         <v>8</v>
       </c>
       <c r="H619" t="n">
-        <v>0.01293670851737261</v>
+        <v>0.01146640721708536</v>
       </c>
     </row>
     <row r="620">
@@ -19037,7 +19037,7 @@
         <v>4</v>
       </c>
       <c r="H620" t="n">
-        <v>0.184357687830925</v>
+        <v>0.09439103305339813</v>
       </c>
     </row>
     <row r="621">
@@ -19067,7 +19067,7 @@
         <v>7</v>
       </c>
       <c r="H621" t="n">
-        <v>0.3910426497459412</v>
+        <v>0.4104130566120148</v>
       </c>
     </row>
     <row r="622">
@@ -19097,7 +19097,7 @@
         <v>8</v>
       </c>
       <c r="H622" t="n">
-        <v>0.1220882833003998</v>
+        <v>0.09084701538085938</v>
       </c>
     </row>
     <row r="623">
@@ -19127,7 +19127,7 @@
         <v>24</v>
       </c>
       <c r="H623" t="n">
-        <v>0.7570326924324036</v>
+        <v>0.8241425156593323</v>
       </c>
     </row>
     <row r="624">
@@ -19157,7 +19157,7 @@
         <v>5</v>
       </c>
       <c r="H624" t="n">
-        <v>0.03398695215582848</v>
+        <v>0.04786061868071556</v>
       </c>
     </row>
     <row r="625">
@@ -19187,7 +19187,7 @@
         <v>1</v>
       </c>
       <c r="H625" t="n">
-        <v>0.02350889891386032</v>
+        <v>0.05485016107559204</v>
       </c>
     </row>
     <row r="626">
@@ -19217,7 +19217,7 @@
         <v>14</v>
       </c>
       <c r="H626" t="n">
-        <v>0.5623067021369934</v>
+        <v>0.4646740257740021</v>
       </c>
     </row>
     <row r="627">
@@ -19247,7 +19247,7 @@
         <v>14</v>
       </c>
       <c r="H627" t="n">
-        <v>0.5327526926994324</v>
+        <v>0.3848895728588104</v>
       </c>
     </row>
     <row r="628">
@@ -19277,7 +19277,7 @@
         <v>8</v>
       </c>
       <c r="H628" t="n">
-        <v>0.08238054066896439</v>
+        <v>0.0438748225569725</v>
       </c>
     </row>
     <row r="629">
@@ -19307,7 +19307,7 @@
         <v>5</v>
       </c>
       <c r="H629" t="n">
-        <v>0.1202368587255478</v>
+        <v>0.0537891611456871</v>
       </c>
     </row>
   </sheetData>

</xml_diff>